<commit_message>
Added new RDF data schemes and visual schemes for education-table33-36, fixed XLSX spreadsheets for education-table33-35
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/education-table33.xlsx
+++ b/sources/table_normalization/xlsx/education-table33.xlsx
@@ -649,7 +649,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -667,92 +667,162 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -760,120 +830,65 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="15" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="16" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="18" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="19" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="20" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="6" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="24" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="10" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="11" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="12" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1384,12 +1399,12 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="42" t="s">
+      <c r="L1" s="64" t="s">
         <v>0</v>
       </c>
-      <c r="M1" s="42"/>
-      <c r="N1" s="42"/>
-      <c r="O1" s="42"/>
+      <c r="M1" s="64"/>
+      <c r="N1" s="64"/>
+      <c r="O1" s="64"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1403,45 +1418,45 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="15.5">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="38" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="39"/>
+      <c r="C2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
+      <c r="D2" s="40"/>
+      <c r="E2" s="40"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
       <c r="I2" s="6"/>
-      <c r="J2" s="60" t="s">
+      <c r="J2" s="39" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="M2" s="8" t="s">
+      <c r="K2" s="39"/>
+      <c r="L2" s="39"/>
+      <c r="M2" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
+      <c r="N2" s="40"/>
+      <c r="O2" s="40"/>
+      <c r="P2" s="40"/>
       <c r="Q2" s="6"/>
-      <c r="R2" s="60" t="s">
+      <c r="R2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="S2" s="60"/>
-      <c r="T2" s="43" t="s">
+      <c r="S2" s="39"/>
+      <c r="T2" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="U2" s="43"/>
+      <c r="U2" s="41"/>
       <c r="V2" s="6"/>
-      <c r="W2" s="60" t="s">
+      <c r="W2" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="X2" s="60"/>
-      <c r="Y2" s="44">
+      <c r="X2" s="39"/>
+      <c r="Y2" s="7">
         <v>1</v>
       </c>
       <c r="Z2" s="1"/>
@@ -1475,538 +1490,538 @@
       <c r="Z3" s="1"/>
     </row>
     <row r="4" spans="1:26">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="46"/>
-      <c r="C4" s="38" t="s">
+      <c r="B4" s="48"/>
+      <c r="C4" s="58" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="38"/>
-      <c r="E4" s="38"/>
-      <c r="F4" s="38" t="s">
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="38"/>
-      <c r="H4" s="38"/>
-      <c r="I4" s="38" t="s">
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="38"/>
-      <c r="K4" s="38"/>
-      <c r="L4" s="49" t="s">
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="45" t="s">
         <v>12</v>
       </c>
-      <c r="M4" s="50" t="s">
+      <c r="M4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="O4" s="52" t="s">
+      <c r="N4" s="52"/>
+      <c r="O4" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="P4" s="52"/>
-      <c r="Q4" s="36" t="s">
+      <c r="P4" s="57"/>
+      <c r="Q4" s="60" t="s">
         <v>9</v>
       </c>
-      <c r="R4" s="36"/>
-      <c r="S4" s="36"/>
-      <c r="T4" s="36"/>
-      <c r="U4" s="36" t="s">
+      <c r="R4" s="60"/>
+      <c r="S4" s="60"/>
+      <c r="T4" s="60"/>
+      <c r="U4" s="60" t="s">
         <v>10</v>
       </c>
-      <c r="V4" s="36"/>
-      <c r="W4" s="36"/>
-      <c r="X4" s="36" t="s">
+      <c r="V4" s="60"/>
+      <c r="W4" s="60"/>
+      <c r="X4" s="60" t="s">
         <v>11</v>
       </c>
-      <c r="Y4" s="36"/>
-      <c r="Z4" s="40"/>
+      <c r="Y4" s="60"/>
+      <c r="Z4" s="62"/>
     </row>
     <row r="5" spans="1:26">
-      <c r="A5" s="47"/>
-      <c r="B5" s="48"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
-      <c r="K5" s="39"/>
-      <c r="L5" s="53"/>
-      <c r="M5" s="54"/>
-      <c r="N5" s="55"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="56"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
-      <c r="S5" s="37"/>
-      <c r="T5" s="37"/>
-      <c r="U5" s="37"/>
-      <c r="V5" s="37"/>
-      <c r="W5" s="37"/>
-      <c r="X5" s="37"/>
-      <c r="Y5" s="37"/>
-      <c r="Z5" s="41"/>
+      <c r="A5" s="49"/>
+      <c r="B5" s="50"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
+      <c r="E5" s="59"/>
+      <c r="F5" s="59"/>
+      <c r="G5" s="59"/>
+      <c r="H5" s="59"/>
+      <c r="I5" s="59"/>
+      <c r="J5" s="59"/>
+      <c r="K5" s="59"/>
+      <c r="L5" s="46"/>
+      <c r="M5" s="53"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="61"/>
+      <c r="R5" s="61"/>
+      <c r="S5" s="61"/>
+      <c r="T5" s="61"/>
+      <c r="U5" s="61"/>
+      <c r="V5" s="61"/>
+      <c r="W5" s="61"/>
+      <c r="X5" s="61"/>
+      <c r="Y5" s="61"/>
+      <c r="Z5" s="63"/>
     </row>
     <row r="6" spans="1:26" ht="41" customHeight="1">
-      <c r="A6" s="47"/>
-      <c r="B6" s="48"/>
-      <c r="C6" s="61" t="s">
+      <c r="A6" s="49"/>
+      <c r="B6" s="50"/>
+      <c r="C6" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="56" t="s">
+      <c r="D6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="61" t="s">
+      <c r="E6" s="8"/>
+      <c r="F6" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="G6" s="56" t="s">
+      <c r="G6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="56"/>
-      <c r="I6" s="61" t="s">
+      <c r="H6" s="8"/>
+      <c r="I6" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="J6" s="56" t="s">
+      <c r="J6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="K6" s="56"/>
-      <c r="L6" s="53"/>
-      <c r="M6" s="54"/>
-      <c r="N6" s="55"/>
-      <c r="O6" s="56"/>
-      <c r="P6" s="56"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="37"/>
-      <c r="S6" s="37"/>
-      <c r="T6" s="37"/>
-      <c r="U6" s="37"/>
-      <c r="V6" s="37"/>
-      <c r="W6" s="37"/>
-      <c r="X6" s="37"/>
-      <c r="Y6" s="37"/>
-      <c r="Z6" s="41"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="53"/>
+      <c r="N6" s="54"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="61"/>
+      <c r="R6" s="61"/>
+      <c r="S6" s="61"/>
+      <c r="T6" s="61"/>
+      <c r="U6" s="61"/>
+      <c r="V6" s="61"/>
+      <c r="W6" s="61"/>
+      <c r="X6" s="61"/>
+      <c r="Y6" s="61"/>
+      <c r="Z6" s="63"/>
     </row>
     <row r="7" spans="1:26" ht="51" customHeight="1">
-      <c r="A7" s="47"/>
-      <c r="B7" s="48"/>
-      <c r="C7" s="61"/>
-      <c r="D7" s="56"/>
-      <c r="E7" s="56"/>
-      <c r="F7" s="61"/>
-      <c r="G7" s="56"/>
-      <c r="H7" s="56"/>
-      <c r="I7" s="61"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="53"/>
-      <c r="M7" s="57"/>
-      <c r="N7" s="58"/>
-      <c r="O7" s="56"/>
-      <c r="P7" s="56"/>
-      <c r="Q7" s="62" t="s">
+      <c r="A7" s="49"/>
+      <c r="B7" s="50"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="46"/>
+      <c r="M7" s="55"/>
+      <c r="N7" s="56"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="R7" s="62"/>
-      <c r="S7" s="62"/>
-      <c r="T7" s="62"/>
-      <c r="U7" s="62" t="s">
+      <c r="R7" s="42"/>
+      <c r="S7" s="42"/>
+      <c r="T7" s="42"/>
+      <c r="U7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="V7" s="62"/>
-      <c r="W7" s="62"/>
-      <c r="X7" s="62" t="s">
+      <c r="V7" s="42"/>
+      <c r="W7" s="42"/>
+      <c r="X7" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="Y7" s="62"/>
-      <c r="Z7" s="63"/>
+      <c r="Y7" s="42"/>
+      <c r="Z7" s="43"/>
     </row>
     <row r="8" spans="1:26" ht="48" customHeight="1">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="36" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="12"/>
+      <c r="B8" s="37"/>
       <c r="C8" s="3">
         <v>10</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="33">
         <v>5</v>
       </c>
-      <c r="E8" s="13"/>
+      <c r="E8" s="33"/>
       <c r="F8" s="3">
         <v>15</v>
       </c>
-      <c r="G8" s="13">
+      <c r="G8" s="33">
         <v>9</v>
       </c>
-      <c r="H8" s="13"/>
+      <c r="H8" s="33"/>
       <c r="I8" s="3">
         <v>75</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="33">
         <v>0</v>
       </c>
-      <c r="K8" s="13"/>
+      <c r="K8" s="33"/>
       <c r="L8" s="3">
         <v>100</v>
       </c>
-      <c r="M8" s="13">
+      <c r="M8" s="33">
         <v>14</v>
       </c>
-      <c r="N8" s="13"/>
-      <c r="O8" s="72" t="s">
+      <c r="N8" s="33"/>
+      <c r="O8" s="65" t="s">
         <v>18</v>
       </c>
-      <c r="P8" s="73"/>
+      <c r="P8" s="66"/>
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
       <c r="T8" s="14"/>
-      <c r="U8" s="9"/>
-      <c r="V8" s="9"/>
-      <c r="W8" s="9"/>
-      <c r="X8" s="9"/>
-      <c r="Y8" s="9"/>
-      <c r="Z8" s="10"/>
+      <c r="U8" s="17"/>
+      <c r="V8" s="17"/>
+      <c r="W8" s="17"/>
+      <c r="X8" s="17"/>
+      <c r="Y8" s="17"/>
+      <c r="Z8" s="18"/>
     </row>
     <row r="9" spans="1:26" ht="18.5">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B9" s="16"/>
+      <c r="B9" s="25"/>
       <c r="C9" s="3">
         <v>10</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="33">
         <v>6</v>
       </c>
-      <c r="E9" s="13"/>
+      <c r="E9" s="33"/>
       <c r="F9" s="3">
         <v>15</v>
       </c>
-      <c r="G9" s="13">
+      <c r="G9" s="33">
         <v>7</v>
       </c>
-      <c r="H9" s="13"/>
+      <c r="H9" s="33"/>
       <c r="I9" s="3">
         <v>75</v>
       </c>
-      <c r="J9" s="13">
+      <c r="J9" s="33">
         <v>0</v>
       </c>
-      <c r="K9" s="13"/>
+      <c r="K9" s="33"/>
       <c r="L9" s="3">
         <v>100</v>
       </c>
-      <c r="M9" s="13">
+      <c r="M9" s="33">
         <v>13</v>
       </c>
-      <c r="N9" s="13"/>
-      <c r="O9" s="74" t="s">
+      <c r="N9" s="33"/>
+      <c r="O9" s="67" t="s">
         <v>20</v>
       </c>
-      <c r="P9" s="74"/>
+      <c r="P9" s="67"/>
       <c r="Q9" s="14"/>
       <c r="R9" s="14"/>
       <c r="S9" s="14"/>
       <c r="T9" s="14"/>
-      <c r="U9" s="9"/>
-      <c r="V9" s="9"/>
-      <c r="W9" s="9"/>
-      <c r="X9" s="9"/>
-      <c r="Y9" s="9"/>
-      <c r="Z9" s="10"/>
+      <c r="U9" s="17"/>
+      <c r="V9" s="17"/>
+      <c r="W9" s="17"/>
+      <c r="X9" s="17"/>
+      <c r="Y9" s="17"/>
+      <c r="Z9" s="18"/>
     </row>
     <row r="10" spans="1:26" ht="18.5">
-      <c r="A10" s="15" t="s">
+      <c r="A10" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B10" s="16"/>
+      <c r="B10" s="25"/>
       <c r="C10" s="3">
         <v>10</v>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="33">
         <v>7</v>
       </c>
-      <c r="E10" s="13"/>
+      <c r="E10" s="33"/>
       <c r="F10" s="3">
         <v>15</v>
       </c>
-      <c r="G10" s="13">
+      <c r="G10" s="33">
         <v>8</v>
       </c>
-      <c r="H10" s="13"/>
+      <c r="H10" s="33"/>
       <c r="I10" s="3">
         <v>75</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="33">
         <v>0</v>
       </c>
-      <c r="K10" s="13"/>
+      <c r="K10" s="33"/>
       <c r="L10" s="3">
         <v>100</v>
       </c>
-      <c r="M10" s="13">
+      <c r="M10" s="33">
         <v>15</v>
       </c>
-      <c r="N10" s="13"/>
-      <c r="O10" s="74" t="s">
+      <c r="N10" s="33"/>
+      <c r="O10" s="67" t="s">
         <v>22</v>
       </c>
-      <c r="P10" s="74"/>
+      <c r="P10" s="67"/>
       <c r="Q10" s="14"/>
       <c r="R10" s="14"/>
       <c r="S10" s="14"/>
       <c r="T10" s="14"/>
-      <c r="U10" s="9"/>
-      <c r="V10" s="9"/>
-      <c r="W10" s="9"/>
-      <c r="X10" s="9"/>
-      <c r="Y10" s="9"/>
-      <c r="Z10" s="10"/>
+      <c r="U10" s="17"/>
+      <c r="V10" s="17"/>
+      <c r="W10" s="17"/>
+      <c r="X10" s="17"/>
+      <c r="Y10" s="17"/>
+      <c r="Z10" s="18"/>
     </row>
     <row r="11" spans="1:26" ht="18.5">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="16"/>
+      <c r="B11" s="25"/>
       <c r="C11" s="3">
         <v>10</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="33">
         <v>9</v>
       </c>
-      <c r="E11" s="13"/>
+      <c r="E11" s="33"/>
       <c r="F11" s="3">
         <v>15</v>
       </c>
-      <c r="G11" s="13">
+      <c r="G11" s="33">
         <v>8</v>
       </c>
-      <c r="H11" s="13"/>
+      <c r="H11" s="33"/>
       <c r="I11" s="3">
         <v>75</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="33">
         <v>0</v>
       </c>
-      <c r="K11" s="13"/>
+      <c r="K11" s="33"/>
       <c r="L11" s="3">
         <v>100</v>
       </c>
-      <c r="M11" s="13">
+      <c r="M11" s="33">
         <v>17</v>
       </c>
-      <c r="N11" s="13"/>
-      <c r="O11" s="74" t="s">
+      <c r="N11" s="33"/>
+      <c r="O11" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="P11" s="74"/>
+      <c r="P11" s="67"/>
       <c r="Q11" s="14"/>
       <c r="R11" s="14"/>
       <c r="S11" s="14"/>
       <c r="T11" s="14"/>
-      <c r="U11" s="9"/>
-      <c r="V11" s="9"/>
-      <c r="W11" s="9"/>
-      <c r="X11" s="9"/>
-      <c r="Y11" s="9"/>
-      <c r="Z11" s="10"/>
+      <c r="U11" s="17"/>
+      <c r="V11" s="17"/>
+      <c r="W11" s="17"/>
+      <c r="X11" s="17"/>
+      <c r="Y11" s="17"/>
+      <c r="Z11" s="18"/>
     </row>
     <row r="12" spans="1:26" ht="18.5">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="16"/>
+      <c r="B12" s="25"/>
       <c r="C12" s="3">
         <v>10</v>
       </c>
-      <c r="D12" s="13">
+      <c r="D12" s="33">
         <v>9</v>
       </c>
-      <c r="E12" s="13"/>
+      <c r="E12" s="33"/>
       <c r="F12" s="3">
         <v>15</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="33">
         <v>8</v>
       </c>
-      <c r="H12" s="13"/>
+      <c r="H12" s="33"/>
       <c r="I12" s="3">
         <v>75</v>
       </c>
-      <c r="J12" s="13">
+      <c r="J12" s="33">
         <v>0</v>
       </c>
-      <c r="K12" s="13"/>
+      <c r="K12" s="33"/>
       <c r="L12" s="3">
         <v>100</v>
       </c>
-      <c r="M12" s="13">
+      <c r="M12" s="33">
         <v>17</v>
       </c>
-      <c r="N12" s="13"/>
-      <c r="O12" s="74" t="s">
+      <c r="N12" s="33"/>
+      <c r="O12" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="P12" s="74"/>
+      <c r="P12" s="67"/>
       <c r="Q12" s="14"/>
       <c r="R12" s="14"/>
       <c r="S12" s="14"/>
       <c r="T12" s="14"/>
-      <c r="U12" s="9"/>
-      <c r="V12" s="9"/>
-      <c r="W12" s="9"/>
-      <c r="X12" s="9"/>
-      <c r="Y12" s="9"/>
-      <c r="Z12" s="10"/>
+      <c r="U12" s="17"/>
+      <c r="V12" s="17"/>
+      <c r="W12" s="17"/>
+      <c r="X12" s="17"/>
+      <c r="Y12" s="17"/>
+      <c r="Z12" s="18"/>
     </row>
     <row r="13" spans="1:26" ht="34" customHeight="1">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B13" s="16"/>
+      <c r="B13" s="25"/>
       <c r="C13" s="3">
         <v>10</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D13" s="33">
         <v>6</v>
       </c>
-      <c r="E13" s="13"/>
+      <c r="E13" s="33"/>
       <c r="F13" s="3">
         <v>15</v>
       </c>
-      <c r="G13" s="13">
+      <c r="G13" s="33">
         <v>7</v>
       </c>
-      <c r="H13" s="13"/>
+      <c r="H13" s="33"/>
       <c r="I13" s="3">
         <v>75</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="33">
         <v>0</v>
       </c>
-      <c r="K13" s="13"/>
+      <c r="K13" s="33"/>
       <c r="L13" s="3">
         <v>100</v>
       </c>
-      <c r="M13" s="13">
+      <c r="M13" s="33">
         <v>13</v>
       </c>
-      <c r="N13" s="13"/>
-      <c r="O13" s="74" t="s">
+      <c r="N13" s="33"/>
+      <c r="O13" s="67" t="s">
         <v>28</v>
       </c>
-      <c r="P13" s="74"/>
+      <c r="P13" s="67"/>
       <c r="Q13" s="14"/>
       <c r="R13" s="14"/>
       <c r="S13" s="14"/>
       <c r="T13" s="14"/>
-      <c r="U13" s="9"/>
-      <c r="V13" s="9"/>
-      <c r="W13" s="9"/>
-      <c r="X13" s="9"/>
-      <c r="Y13" s="9"/>
-      <c r="Z13" s="10"/>
+      <c r="U13" s="17"/>
+      <c r="V13" s="17"/>
+      <c r="W13" s="17"/>
+      <c r="X13" s="17"/>
+      <c r="Y13" s="17"/>
+      <c r="Z13" s="18"/>
     </row>
     <row r="14" spans="1:26" ht="18.5">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B14" s="16"/>
+      <c r="B14" s="25"/>
       <c r="C14" s="4"/>
-      <c r="D14" s="13"/>
-      <c r="E14" s="13"/>
+      <c r="D14" s="33"/>
+      <c r="E14" s="33"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="17"/>
-      <c r="H14" s="18"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="35"/>
       <c r="I14" s="4"/>
-      <c r="J14" s="13"/>
-      <c r="K14" s="13"/>
+      <c r="J14" s="33"/>
+      <c r="K14" s="33"/>
       <c r="L14" s="4">
         <v>0</v>
       </c>
-      <c r="M14" s="13">
+      <c r="M14" s="33">
         <v>0</v>
       </c>
-      <c r="N14" s="13"/>
-      <c r="O14" s="67"/>
-      <c r="P14" s="67"/>
+      <c r="N14" s="33"/>
+      <c r="O14" s="68"/>
+      <c r="P14" s="68"/>
       <c r="Q14" s="14"/>
       <c r="R14" s="14"/>
       <c r="S14" s="14"/>
       <c r="T14" s="14"/>
-      <c r="U14" s="9"/>
-      <c r="V14" s="9"/>
-      <c r="W14" s="9"/>
-      <c r="X14" s="9"/>
-      <c r="Y14" s="9"/>
-      <c r="Z14" s="10"/>
+      <c r="U14" s="17"/>
+      <c r="V14" s="17"/>
+      <c r="W14" s="17"/>
+      <c r="X14" s="17"/>
+      <c r="Y14" s="17"/>
+      <c r="Z14" s="18"/>
     </row>
     <row r="15" spans="1:26" ht="35" customHeight="1">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B15" s="16"/>
+      <c r="B15" s="23"/>
       <c r="C15" s="5">
         <v>60</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="26">
         <v>42</v>
       </c>
-      <c r="E15" s="20"/>
+      <c r="E15" s="27"/>
       <c r="F15" s="5">
         <v>90</v>
       </c>
-      <c r="G15" s="19">
+      <c r="G15" s="26">
         <v>47</v>
       </c>
-      <c r="H15" s="20"/>
+      <c r="H15" s="27"/>
       <c r="I15" s="5">
         <v>450</v>
       </c>
-      <c r="J15" s="19">
+      <c r="J15" s="26">
         <v>0</v>
       </c>
-      <c r="K15" s="20"/>
-      <c r="L15" s="7">
+      <c r="K15" s="27"/>
+      <c r="L15" s="80">
         <v>600</v>
       </c>
-      <c r="M15" s="21">
+      <c r="M15" s="81">
         <v>89</v>
       </c>
-      <c r="N15" s="21"/>
-      <c r="O15" s="75" t="s">
+      <c r="N15" s="81"/>
+      <c r="O15" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="P15" s="76"/>
-      <c r="Q15" s="22" t="s">
+      <c r="P15" s="29"/>
+      <c r="Q15" s="30" t="s">
         <v>32</v>
       </c>
-      <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
-      <c r="T15" s="24"/>
-      <c r="U15" s="9"/>
-      <c r="V15" s="9"/>
-      <c r="W15" s="9"/>
-      <c r="X15" s="9"/>
-      <c r="Y15" s="9"/>
-      <c r="Z15" s="10"/>
+      <c r="R15" s="31"/>
+      <c r="S15" s="31"/>
+      <c r="T15" s="32"/>
+      <c r="U15" s="17"/>
+      <c r="V15" s="17"/>
+      <c r="W15" s="17"/>
+      <c r="X15" s="17"/>
+      <c r="Y15" s="17"/>
+      <c r="Z15" s="18"/>
     </row>
     <row r="16" spans="1:26">
-      <c r="A16" s="64" t="s">
+      <c r="A16" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="B16" s="65"/>
+      <c r="B16" s="74"/>
       <c r="C16" s="2"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
       <c r="F16" s="2"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="26"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="16"/>
       <c r="I16" s="2"/>
       <c r="J16" s="14"/>
       <c r="K16" s="14"/>
@@ -2019,18 +2034,18 @@
       <c r="R16" s="14"/>
       <c r="S16" s="14"/>
       <c r="T16" s="14"/>
-      <c r="U16" s="9"/>
-      <c r="V16" s="9"/>
-      <c r="W16" s="9"/>
-      <c r="X16" s="9"/>
-      <c r="Y16" s="9"/>
-      <c r="Z16" s="10"/>
+      <c r="U16" s="17"/>
+      <c r="V16" s="17"/>
+      <c r="W16" s="17"/>
+      <c r="X16" s="17"/>
+      <c r="Y16" s="17"/>
+      <c r="Z16" s="18"/>
     </row>
     <row r="17" spans="1:26" ht="21">
-      <c r="A17" s="66" t="s">
+      <c r="A17" s="75" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="67"/>
+      <c r="B17" s="76"/>
       <c r="C17" s="14"/>
       <c r="D17" s="14"/>
       <c r="E17" s="14"/>
@@ -2040,31 +2055,31 @@
       <c r="I17" s="14"/>
       <c r="J17" s="14"/>
       <c r="K17" s="14"/>
-      <c r="L17" s="27" t="s">
+      <c r="L17" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="M17" s="28"/>
-      <c r="N17" s="29"/>
-      <c r="O17" s="27" t="s">
+      <c r="M17" s="78"/>
+      <c r="N17" s="79"/>
+      <c r="O17" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="P17" s="28"/>
-      <c r="Q17" s="28"/>
-      <c r="R17" s="28"/>
-      <c r="S17" s="28"/>
-      <c r="T17" s="28"/>
-      <c r="U17" s="28"/>
-      <c r="V17" s="28"/>
-      <c r="W17" s="28"/>
-      <c r="X17" s="28"/>
-      <c r="Y17" s="28"/>
-      <c r="Z17" s="30"/>
+      <c r="P17" s="20"/>
+      <c r="Q17" s="20"/>
+      <c r="R17" s="20"/>
+      <c r="S17" s="20"/>
+      <c r="T17" s="20"/>
+      <c r="U17" s="20"/>
+      <c r="V17" s="20"/>
+      <c r="W17" s="20"/>
+      <c r="X17" s="20"/>
+      <c r="Y17" s="20"/>
+      <c r="Z17" s="21"/>
     </row>
     <row r="18" spans="1:26">
-      <c r="A18" s="68" t="s">
+      <c r="A18" s="69" t="s">
         <v>37</v>
       </c>
-      <c r="B18" s="69"/>
+      <c r="B18" s="70"/>
       <c r="C18" s="14"/>
       <c r="D18" s="14"/>
       <c r="E18" s="14"/>
@@ -2077,24 +2092,24 @@
       <c r="L18" s="14"/>
       <c r="M18" s="14"/>
       <c r="N18" s="14"/>
-      <c r="O18" s="25"/>
-      <c r="P18" s="26"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="16"/>
       <c r="Q18" s="14"/>
       <c r="R18" s="14"/>
       <c r="S18" s="14"/>
       <c r="T18" s="14"/>
-      <c r="U18" s="9"/>
-      <c r="V18" s="9"/>
-      <c r="W18" s="9"/>
-      <c r="X18" s="9"/>
-      <c r="Y18" s="9"/>
-      <c r="Z18" s="10"/>
+      <c r="U18" s="17"/>
+      <c r="V18" s="17"/>
+      <c r="W18" s="17"/>
+      <c r="X18" s="17"/>
+      <c r="Y18" s="17"/>
+      <c r="Z18" s="18"/>
     </row>
     <row r="19" spans="1:26">
-      <c r="A19" s="68" t="s">
+      <c r="A19" s="69" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="69"/>
+      <c r="B19" s="70"/>
       <c r="C19" s="14"/>
       <c r="D19" s="14"/>
       <c r="E19" s="14"/>
@@ -2107,168 +2122,51 @@
       <c r="L19" s="14"/>
       <c r="M19" s="14"/>
       <c r="N19" s="14"/>
-      <c r="O19" s="25"/>
-      <c r="P19" s="26"/>
+      <c r="O19" s="15"/>
+      <c r="P19" s="16"/>
       <c r="Q19" s="14"/>
       <c r="R19" s="14"/>
       <c r="S19" s="14"/>
       <c r="T19" s="14"/>
-      <c r="U19" s="9"/>
-      <c r="V19" s="9"/>
-      <c r="W19" s="9"/>
-      <c r="X19" s="9"/>
-      <c r="Y19" s="9"/>
-      <c r="Z19" s="10"/>
+      <c r="U19" s="17"/>
+      <c r="V19" s="17"/>
+      <c r="W19" s="17"/>
+      <c r="X19" s="17"/>
+      <c r="Y19" s="17"/>
+      <c r="Z19" s="18"/>
     </row>
     <row r="20" spans="1:26">
-      <c r="A20" s="70" t="s">
+      <c r="A20" s="71" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="71"/>
-      <c r="C20" s="31"/>
-      <c r="D20" s="31"/>
-      <c r="E20" s="31"/>
-      <c r="F20" s="31"/>
-      <c r="G20" s="31"/>
-      <c r="H20" s="31"/>
-      <c r="I20" s="31"/>
-      <c r="J20" s="31"/>
-      <c r="K20" s="31"/>
-      <c r="L20" s="31"/>
-      <c r="M20" s="31"/>
-      <c r="N20" s="31"/>
-      <c r="O20" s="32"/>
-      <c r="P20" s="33"/>
-      <c r="Q20" s="31"/>
-      <c r="R20" s="31"/>
-      <c r="S20" s="31"/>
-      <c r="T20" s="31"/>
-      <c r="U20" s="34"/>
-      <c r="V20" s="34"/>
-      <c r="W20" s="34"/>
-      <c r="X20" s="34"/>
-      <c r="Y20" s="34"/>
-      <c r="Z20" s="35"/>
+      <c r="B20" s="72"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="10"/>
+      <c r="P20" s="11"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" s="9"/>
+      <c r="T20" s="9"/>
+      <c r="U20" s="12"/>
+      <c r="V20" s="12"/>
+      <c r="W20" s="12"/>
+      <c r="X20" s="12"/>
+      <c r="Y20" s="12"/>
+      <c r="Z20" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="141">
-    <mergeCell ref="D6:E7"/>
-    <mergeCell ref="J6:K7"/>
-    <mergeCell ref="G6:H7"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="I20:K20"/>
-    <mergeCell ref="L20:N20"/>
-    <mergeCell ref="O20:P20"/>
-    <mergeCell ref="Q20:T20"/>
-    <mergeCell ref="U20:W20"/>
-    <mergeCell ref="X20:Z20"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="I19:K19"/>
-    <mergeCell ref="L19:N19"/>
-    <mergeCell ref="O19:P19"/>
-    <mergeCell ref="Q19:T19"/>
-    <mergeCell ref="U19:W19"/>
-    <mergeCell ref="X19:Z19"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:E17"/>
-    <mergeCell ref="F17:H17"/>
-    <mergeCell ref="I17:K17"/>
-    <mergeCell ref="L17:N17"/>
-    <mergeCell ref="O17:Z17"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="C18:E18"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="I18:K18"/>
-    <mergeCell ref="L18:N18"/>
-    <mergeCell ref="O18:P18"/>
-    <mergeCell ref="Q18:T18"/>
-    <mergeCell ref="U18:W18"/>
-    <mergeCell ref="X18:Z18"/>
-    <mergeCell ref="A16:B16"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="J16:K16"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="Q16:T16"/>
-    <mergeCell ref="U16:W16"/>
-    <mergeCell ref="X16:Z16"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="Q15:T15"/>
-    <mergeCell ref="U15:W15"/>
-    <mergeCell ref="X15:Z15"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="Q14:T14"/>
-    <mergeCell ref="U14:W14"/>
-    <mergeCell ref="X14:Z14"/>
-    <mergeCell ref="A13:B13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="M13:N13"/>
-    <mergeCell ref="O13:P13"/>
-    <mergeCell ref="Q13:T13"/>
-    <mergeCell ref="U13:W13"/>
-    <mergeCell ref="X13:Z13"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="O12:P12"/>
-    <mergeCell ref="Q12:T12"/>
-    <mergeCell ref="U12:W12"/>
-    <mergeCell ref="X12:Z12"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="O11:P11"/>
-    <mergeCell ref="Q11:T11"/>
-    <mergeCell ref="U11:W11"/>
-    <mergeCell ref="X11:Z11"/>
-    <mergeCell ref="A10:B10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="J10:K10"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="O10:P10"/>
-    <mergeCell ref="Q10:T10"/>
-    <mergeCell ref="U10:W10"/>
-    <mergeCell ref="X10:Z10"/>
-    <mergeCell ref="A9:B9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="M9:N9"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="Q9:T9"/>
-    <mergeCell ref="U9:W9"/>
-    <mergeCell ref="X9:Z9"/>
-    <mergeCell ref="A8:B8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="G8:H8"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="M8:N8"/>
-    <mergeCell ref="O8:P8"/>
-    <mergeCell ref="Q8:T8"/>
-    <mergeCell ref="U8:W8"/>
-    <mergeCell ref="X8:Z8"/>
     <mergeCell ref="L1:O1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C2:H2"/>
@@ -2293,6 +2191,123 @@
     <mergeCell ref="Q4:T6"/>
     <mergeCell ref="U4:W6"/>
     <mergeCell ref="X4:Z6"/>
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="G8:H8"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="M8:N8"/>
+    <mergeCell ref="O8:P8"/>
+    <mergeCell ref="Q8:T8"/>
+    <mergeCell ref="U8:W8"/>
+    <mergeCell ref="X8:Z8"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="M9:N9"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="Q9:T9"/>
+    <mergeCell ref="U9:W9"/>
+    <mergeCell ref="X9:Z9"/>
+    <mergeCell ref="A10:B10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="J10:K10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="O10:P10"/>
+    <mergeCell ref="Q10:T10"/>
+    <mergeCell ref="U10:W10"/>
+    <mergeCell ref="X10:Z10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="O11:P11"/>
+    <mergeCell ref="Q11:T11"/>
+    <mergeCell ref="U11:W11"/>
+    <mergeCell ref="X11:Z11"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="G12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="O12:P12"/>
+    <mergeCell ref="Q12:T12"/>
+    <mergeCell ref="U12:W12"/>
+    <mergeCell ref="X12:Z12"/>
+    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="M13:N13"/>
+    <mergeCell ref="O13:P13"/>
+    <mergeCell ref="Q13:T13"/>
+    <mergeCell ref="U13:W13"/>
+    <mergeCell ref="X13:Z13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="Q14:T14"/>
+    <mergeCell ref="U14:W14"/>
+    <mergeCell ref="X14:Z14"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="Q15:T15"/>
+    <mergeCell ref="U15:W15"/>
+    <mergeCell ref="X15:Z15"/>
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="J16:K16"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="Q16:T16"/>
+    <mergeCell ref="U16:W16"/>
+    <mergeCell ref="X16:Z16"/>
+    <mergeCell ref="Q20:T20"/>
+    <mergeCell ref="U20:W20"/>
+    <mergeCell ref="X20:Z20"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="F19:H19"/>
+    <mergeCell ref="I19:K19"/>
+    <mergeCell ref="L19:N19"/>
+    <mergeCell ref="O19:P19"/>
+    <mergeCell ref="Q19:T19"/>
+    <mergeCell ref="U19:W19"/>
+    <mergeCell ref="X19:Z19"/>
+    <mergeCell ref="D6:E7"/>
+    <mergeCell ref="J6:K7"/>
+    <mergeCell ref="G6:H7"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="F20:H20"/>
+    <mergeCell ref="I20:K20"/>
+    <mergeCell ref="L20:N20"/>
+    <mergeCell ref="O20:P20"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="F17:H17"/>
+    <mergeCell ref="I17:K17"/>
+    <mergeCell ref="L17:N17"/>
+    <mergeCell ref="O17:Z17"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="I18:K18"/>
+    <mergeCell ref="L18:N18"/>
+    <mergeCell ref="O18:P18"/>
+    <mergeCell ref="Q18:T18"/>
+    <mergeCell ref="U18:W18"/>
+    <mergeCell ref="X18:Z18"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T2:U2">

</xml_diff>